<commit_message>
changed names of pam components
</commit_message>
<xml_diff>
--- a/ligament&muscle_lengths.xlsx
+++ b/ligament&muscle_lengths.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Tokyo Tech\Project\Dog Robot\OpenSim Model\Hoshiramu_robot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4f506518823dc09/Tokyo Tech/Project/Dog Robot/OpenSim Model/Hoshiramu_robot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="113_{2F044B86-E1F1-48E8-947D-222534BCA949}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{A3720308-5D8D-4A73-BF4F-5F9F19E53F2C}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="113_{2F044B86-E1F1-48E8-947D-222534BCA949}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{C7D35074-89A7-4A66-911F-130D3E022D36}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" xr2:uid="{26156378-0049-4A8B-8CB0-3F3BBDC12CF9}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2" xr2:uid="{26156378-0049-4A8B-8CB0-3F3BBDC12CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Ligaments" sheetId="1" r:id="rId1"/>
     <sheet name="Muscles(L)" sheetId="2" r:id="rId2"/>
+    <sheet name="Tendons(L)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="22">
   <si>
     <t>stf_L</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -901,4 +902,233 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB99F533-89CE-4002-A23E-0EB847934D80}">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <f>0+6</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <f>0+15</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <f>0+10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <f>0+10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <f>0+10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <f>0+10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <f>0+10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <f>10+20</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <f>35+65</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>